<commit_message>
trends-landing hero: keep only the primary "See trends" CTA
The source hero carries two CTAs (See trends + Explore the blog); this page
should show only "See trends". Drop the secondary hero CTA in a page-scoped
pre-parse step in import-trends-landing.js (scoped to the hero header's button
group so the shared columns-feature parser and other pages are unaffected;
idempotent — keeps only the first anchor).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-trends-landing.report.xlsx
+++ b/tools/importer/reports/import-trends-landing.report.xlsx
@@ -70,7 +70,7 @@
     <t>article-index</t>
   </si>
   <si>
-    <t>2026-09-02T20:50:53.168Z</t>
+    <t>2026-09-03T05:19:03.131Z</t>
   </si>
   <si>
     <t>Blog — WKND Trendsetters</t>
@@ -106,7 +106,7 @@
     <t>trends-landing</t>
   </si>
   <si>
-    <t>2026-09-03T05:18:58.003Z</t>
+    <t>2026-09-03T05:46:00.231Z</t>
   </si>
   <si>
     <t>Fashion Trends for Young Adults - Fashion Blog</t>

</xml_diff>